<commit_message>
Spec de análises extras terminadas
</commit_message>
<xml_diff>
--- a/relatorios_referencia/bandeirante/perfil_estatistico_anual.xlsx
+++ b/relatorios_referencia/bandeirante/perfil_estatistico_anual.xlsx
@@ -9256,7 +9256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9553,6 +9553,23 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>regra</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>sem as Taxas TEIFa Oper e TEIP Oper no nível da usina</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>